<commit_message>
Atualizacao Monitor (upload web) - publicacao manual apos falha no script
</commit_message>
<xml_diff>
--- a/data/mensal_status/manuais_cache.xlsx
+++ b/data/mensal_status/manuais_cache.xlsx
@@ -387,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -852,6 +852,20 @@
         <v>70</v>
       </c>
     </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="2">
+        <v>46252</v>
+      </c>
+      <c r="B34">
+        <v>609</v>
+      </c>
+      <c r="C34">
+        <v>604</v>
+      </c>
+      <c r="D34">
+        <v>586</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>